<commit_message>
Fix the three design-patent links in the vigilance file.
Google Patents only opens those records when the URL ends in S1, matching the corrected workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/docs/afc-destaflex.xlsx
+++ b/public/docs/afc-destaflex.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimilitareduco-my.sharepoint.com/personal/est_javiere_perez_unimilitar_edu_co/Documents/Documents/documentos de la universidad/cnc/javier enmanuel perez millan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A739F151-64EE-4599-A384-6D73EBB74607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9847ABD0-4940-4861-8A19-323F941C91BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -293,9 +293,6 @@
     <t>Al ser una patente de diseño, protege únicamente la apariencia estética exterior y no la mecánica interna.</t>
   </si>
   <si>
-    <t>https://patents.google.com/patent/USD562658S/en</t>
-  </si>
-  <si>
     <t>US D962,030 S</t>
   </si>
   <si>
@@ -314,9 +311,6 @@
     <t>Ámbito de aplicación limitado a botellas con chapa o cápsula de vino.</t>
   </si>
   <si>
-    <t>https://patents.google.com/patent/USD962030S/en</t>
-  </si>
-  <si>
     <t>US D726,517 S</t>
   </si>
   <si>
@@ -335,9 +329,6 @@
     <t>Ofrece un brazo de palanca menor al destapar botellas en comparación con abrebotellas de mango largo.</t>
   </si>
   <si>
-    <t>https://patents.google.com/patent/USD726517S/en</t>
-  </si>
-  <si>
     <t>CN 210103421 U</t>
   </si>
   <si>
@@ -990,13 +981,22 @@
   </si>
   <si>
     <t>US$ 1.095 millones. (2025)</t>
+  </si>
+  <si>
+    <t>https://patents.google.com/patent/USD562658S1/en</t>
+  </si>
+  <si>
+    <t>https://patents.google.com/patent/USD962030S1/en</t>
+  </si>
+  <si>
+    <t>https://patents.google.com/patent/USD726517S1/en</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1017,6 +1017,14 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1241,10 +1249,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1255,36 +1264,40 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2226,183 +2239,187 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="16" t="s">
+      <c r="C2" s="6"/>
+      <c r="D2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="11"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="6"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B3" s="14"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="15"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="9"/>
     </row>
     <row r="4" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="19" t="s">
+      <c r="C4" s="6"/>
+      <c r="D4" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="21"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="15"/>
     </row>
     <row r="5" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="12"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="7" t="s">
+      <c r="B5" s="17"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="9"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="12"/>
     </row>
     <row r="6" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="12"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="7" t="s">
+      <c r="B6" s="17"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="9"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="12"/>
     </row>
     <row r="7" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="12"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="7" t="s">
+      <c r="B7" s="17"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="9"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="12"/>
     </row>
     <row r="8" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="7" t="s">
+      <c r="B8" s="17"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="9"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="12"/>
     </row>
     <row r="9" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="14"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="4" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="6"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21"/>
     </row>
     <row r="10" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="19" t="s">
+      <c r="C10" s="6"/>
+      <c r="D10" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="21"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="15"/>
     </row>
     <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="12"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="7" t="s">
+      <c r="B11" s="17"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="9"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="12"/>
     </row>
     <row r="12" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="12"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="7" t="s">
+      <c r="B12" s="17"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="9"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="12"/>
     </row>
     <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="14"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="4" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="6"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="21"/>
     </row>
     <row r="14" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="19" t="s">
+      <c r="C14" s="6"/>
+      <c r="D14" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="21"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="15"/>
     </row>
     <row r="15" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="12"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="7" t="s">
+      <c r="B15" s="17"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="9"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="12"/>
     </row>
     <row r="16" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="12"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="7" t="s">
+      <c r="B16" s="17"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="9"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="12"/>
     </row>
     <row r="17" spans="2:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="7" t="s">
+      <c r="B17" s="17"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="9"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="12"/>
     </row>
     <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="14"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="4" t="s">
+      <c r="B18" s="7"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="6"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="B10:C13"/>
+    <mergeCell ref="D15:G15"/>
     <mergeCell ref="D2:G3"/>
     <mergeCell ref="D5:G5"/>
     <mergeCell ref="D14:G14"/>
@@ -2419,10 +2436,6 @@
     <mergeCell ref="D4:G4"/>
     <mergeCell ref="D18:G18"/>
     <mergeCell ref="D9:G9"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="B10:C13"/>
-    <mergeCell ref="D15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2599,215 +2612,215 @@
       <c r="F8" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>89</v>
+      <c r="G8" s="22" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>96</v>
+      <c r="G9" s="22" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>103</v>
+      <c r="G10" s="22" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>149</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="210" customHeight="1" x14ac:dyDescent="0.3">
@@ -2818,16 +2831,16 @@
         <v>77</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>82</v>
@@ -2835,13 +2848,13 @@
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>44</v>
@@ -2858,367 +2871,367 @@
     </row>
     <row r="21" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>184</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="G27" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="E29" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="G29" s="2" t="s">
         <v>216</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="F30" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="G30" s="2" t="s">
         <v>223</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D31" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D32" s="2" t="s">
+      <c r="G32" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="E34" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="E35" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="G35" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>262</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>47</v>
@@ -3226,347 +3239,347 @@
     </row>
     <row r="38" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="D38" s="2" t="s">
+      <c r="G38" s="2" t="s">
         <v>264</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>272</v>
-      </c>
       <c r="G39" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="E40" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>277</v>
-      </c>
       <c r="G40" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D41" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>279</v>
-      </c>
       <c r="F41" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>287</v>
-      </c>
       <c r="G43" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>291</v>
-      </c>
       <c r="G44" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D45" s="2" t="s">
+      <c r="G45" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C51" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="D51" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>313</v>
-      </c>
       <c r="G51" s="2" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D52" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="G52" s="2" t="s">
         <v>314</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>